<commit_message>
Update pending Excel files
</commit_message>
<xml_diff>
--- a/Mas กลุ่มสินค้าที่ผลิตได้มากกว่า 1 สายพาน.xlsx
+++ b/Mas กลุ่มสินค้าที่ผลิตได้มากกว่า 1 สายพาน.xlsx
@@ -8,16 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parinya.the\Production-STEP3-Phraputthabath\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B3E5E0-6E1C-4E5C-AE67-107A25E6ABD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F473D36F-E023-4C19-B385-0E0CEF57BAD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mas_group_station_rule" sheetId="1" r:id="rId1"/>
     <sheet name="columns" sheetId="2" r:id="rId2"/>
     <sheet name="split_mode_examples" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -630,7 +643,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K36"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.84375" customWidth="1"/>
     <col min="2" max="2" width="16.84375" customWidth="1"/>
@@ -644,7 +657,7 @@
     <col min="11" max="11" width="120.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -679,7 +692,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -714,7 +727,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -749,7 +762,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -784,7 +797,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -819,7 +832,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -854,7 +867,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -889,7 +902,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -924,7 +937,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -959,7 +972,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -994,7 +1007,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -1029,7 +1042,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -1064,7 +1077,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -1099,7 +1112,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>35</v>
       </c>
@@ -1134,7 +1147,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -1169,7 +1182,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -1204,7 +1217,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -1239,7 +1252,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1274,7 +1287,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -1309,7 +1322,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1344,7 +1357,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -1379,7 +1392,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>30</v>
       </c>
@@ -1414,7 +1427,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -1449,7 +1462,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -1484,7 +1497,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>20</v>
       </c>
@@ -1519,7 +1532,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -1554,7 +1567,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>43</v>
       </c>
@@ -1589,7 +1602,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>44</v>
       </c>
@@ -1624,7 +1637,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>45</v>
       </c>
@@ -1659,7 +1672,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>46</v>
       </c>
@@ -1694,7 +1707,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>47</v>
       </c>
@@ -1729,7 +1742,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -1764,7 +1777,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>27</v>
       </c>
@@ -1799,7 +1812,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>28</v>
       </c>
@@ -1834,7 +1847,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>30</v>
       </c>
@@ -1869,7 +1882,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>48</v>
       </c>
@@ -1906,6 +1919,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="EpmWorksheetKeyString_GUID" r:id="rId1"/>
+  </customProperties>
   <ignoredErrors>
     <ignoredError sqref="A1:K36" numberStoredAsText="1"/>
   </ignoredErrors>
@@ -1915,13 +1931,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.84375" customWidth="1"/>
     <col min="2" max="2" width="100.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>49</v>
       </c>
@@ -1929,7 +1945,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1937,7 +1953,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1945,7 +1961,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1953,7 +1969,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1961,7 +1977,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1969,7 +1985,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1977,7 +1993,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1985,7 +2001,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1993,7 +2009,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -2001,7 +2017,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2009,7 +2025,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -2019,9 +2035,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <customProperties>
-    <customPr name="EpmWorksheetKeyString_GUID" r:id="rId1"/>
-  </customProperties>
   <ignoredErrors>
     <ignoredError sqref="A1:B12" numberStoredAsText="1"/>
   </ignoredErrors>
@@ -2031,14 +2044,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.84375" customWidth="1"/>
     <col min="2" max="2" width="65.84375" customWidth="1"/>
     <col min="3" max="3" width="55.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -2049,7 +2062,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -2060,7 +2073,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -2071,7 +2084,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>68</v>
       </c>
@@ -2082,7 +2095,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -2093,7 +2106,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>74</v>
       </c>

</xml_diff>